<commit_message>
Simplify to DOCX-only output, remove PDF generation
- Remove HTML-based PDF rendering pipeline (extractTemplateInfo, compressImageToDataUrl, renderPdfFromHtml)
- Remove html2canvas and jsPDF CDN dependencies
- Remove render-container div and related CSS
- Remove output format UI and unused output-options CSS
- Single DOCX output per attendee, pixel-perfect from template
</commit_message>
<xml_diff>
--- a/Template Test/BICSI Course Names.xlsx
+++ b/Template Test/BICSI Course Names.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://panduit-my.sharepoint.com/personal/usr091281_panduit_com/Documents/Documents/GitHub Repositories/BICSI Certificat Auto-Fill/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://panduit-my.sharepoint.com/personal/usr091281_panduit_com/Documents/Documents/GitHub Repositories/BICSI Certificat Auto-Fill/Template Test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC104811919D4ABE5ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62607D8E-A840-4A9A-83C8-F8579C76D88E}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_F25DC773A252ABDACC104811919D4ABE5ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F143A62-F1E4-4FF7-882F-3F411E188359}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-3870" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47070" yWindow="-2820" windowWidth="18900" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Full Name</t>
   </si>
@@ -43,6 +43,12 @@
   </si>
   <si>
     <t>March 1 2026</t>
+  </si>
+  <si>
+    <t>Course Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trends in Enterprise | Smart Building </t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20.1328125" customWidth="1"/>
@@ -377,7 +383,7 @@
     <col min="3" max="3" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -385,10 +391,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -396,6 +405,9 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>